<commit_message>
fix(p3): restore printed instruction table rows in workbook 06
</commit_message>
<xml_diff>
--- a/tools/candidates/p3-buyer-negative-20261015/06-zhurnal-peredachi.xlsx
+++ b/tools/candidates/p3-buyer-negative-20261015/06-zhurnal-peredachi.xlsx
@@ -2109,18 +2109,18 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="9" t="s">
         <v>28</v>
       </c>
     </row>

</xml_diff>